<commit_message>
Tutor KPI Sorter Jan26
</commit_message>
<xml_diff>
--- a/Tutor_Concerns.xlsx
+++ b/Tutor_Concerns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tyler_harrington2/Desktop/FL_Dashboards/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5B3D2AC9-73B2-0841-A9CC-D68F5A87B440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{70633AB4-17F6-B142-A387-326E4C698DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{92DEE1D6-509C-344A-AA8F-D8DD2317BD81}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="4137" uniqueCount="602">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5001" uniqueCount="657">
   <si>
     <t>Tutor Name</t>
   </si>
@@ -1842,6 +1842,171 @@
   </si>
   <si>
     <t>11/30/25 - 12/27/25</t>
+  </si>
+  <si>
+    <t>Weighted Repurchases = 0; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Annie Sylvester</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % Sessions on Time &lt; 90%</t>
+  </si>
+  <si>
+    <t>Blake Maly</t>
+  </si>
+  <si>
+    <t>Brittany Drew</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Avg. NPS Score &lt; 8; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Ishita Mehta</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Sessions on Time &lt; 85%; Prep Time % &gt; 15%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>Kira Lioto</t>
+  </si>
+  <si>
+    <t>Krishna Rastogi</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Prep Time % &gt; 15%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Naima Chaudhry</t>
+  </si>
+  <si>
+    <t>Nestor Hernandez</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Noah Robinson</t>
+  </si>
+  <si>
+    <t>Ore Williams</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Rafi Overton</t>
+  </si>
+  <si>
+    <t>Rain Real</t>
+  </si>
+  <si>
+    <t>% Sessions on Time &lt; 85%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Rooa Abdelmagid</t>
+  </si>
+  <si>
+    <t>Saahithi Punnam</t>
+  </si>
+  <si>
+    <t>Scott Greathouse</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % Sessions on Time &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>Syrae Jennings</t>
+  </si>
+  <si>
+    <t>Taryn Parks</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Tina Stegmann</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Weighted Repurchases = 0</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>12/28/25 - 01/24/26</t>
   </si>
 </sst>
 </file>
@@ -2711,7 +2876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA4CB91-83C8-694D-BBCD-170E9881DA10}">
-  <dimension ref="A1:E1034"/>
+  <dimension ref="A1:E1250"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -20295,6 +20460,3678 @@
         <v>600</v>
       </c>
     </row>
+    <row r="1035" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1035" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1035" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1035" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1035">
+        <v>2</v>
+      </c>
+      <c r="E1035" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1036" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1036" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1036" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1036">
+        <v>5</v>
+      </c>
+      <c r="E1036" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1037" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1037" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1037" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1037">
+        <v>2</v>
+      </c>
+      <c r="E1037" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1038" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1038" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1038" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1038">
+        <v>5</v>
+      </c>
+      <c r="E1038" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1039" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1039" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1039" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1039">
+        <v>1</v>
+      </c>
+      <c r="E1039" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1040" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1040" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1040" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1040">
+        <v>2</v>
+      </c>
+      <c r="E1040" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1041" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1041" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1041" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1041">
+        <v>4</v>
+      </c>
+      <c r="E1041" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1042" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1042" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1042" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1042">
+        <v>3</v>
+      </c>
+      <c r="E1042" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1043" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1043" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1043" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1043">
+        <v>4</v>
+      </c>
+      <c r="E1043" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1044" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1044" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1044" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1044">
+        <v>5</v>
+      </c>
+      <c r="E1044" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1045" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1045" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1045">
+        <v>1</v>
+      </c>
+      <c r="E1045" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1046" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1046" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1046">
+        <v>5</v>
+      </c>
+      <c r="E1046" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1047" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1047" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1047" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1047">
+        <v>2</v>
+      </c>
+      <c r="E1047" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1048" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1048" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1048" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1048">
+        <v>4</v>
+      </c>
+      <c r="E1048" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1049" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1049" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1049" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1049">
+        <v>1</v>
+      </c>
+      <c r="E1049" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1050" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1050" t="s">
+        <v>607</v>
+      </c>
+      <c r="C1050" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1050">
+        <v>2</v>
+      </c>
+      <c r="E1050" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1051" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1051" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1051" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1051">
+        <v>2</v>
+      </c>
+      <c r="E1051" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1052" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1052" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1052" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1052">
+        <v>4</v>
+      </c>
+      <c r="E1052" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1053" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1053" t="s">
+        <v>534</v>
+      </c>
+      <c r="C1053" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1053">
+        <v>5</v>
+      </c>
+      <c r="E1053" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1054" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1054" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1054" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1054">
+        <v>2</v>
+      </c>
+      <c r="E1054" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1055" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1055" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1055" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1055">
+        <v>4</v>
+      </c>
+      <c r="E1055" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1056" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1056" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1056" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1056">
+        <v>3</v>
+      </c>
+      <c r="E1056" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1057" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1057" t="s">
+        <v>609</v>
+      </c>
+      <c r="C1057" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1057">
+        <v>3</v>
+      </c>
+      <c r="E1057" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1058" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1058" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1058" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1058">
+        <v>2</v>
+      </c>
+      <c r="E1058" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1059" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1059" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1059" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1059">
+        <v>5</v>
+      </c>
+      <c r="E1059" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1060" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1060" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1060" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1060">
+        <v>2</v>
+      </c>
+      <c r="E1060" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1061" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1061" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1061" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1061">
+        <v>2</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1062" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1062" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1062" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1062">
+        <v>2</v>
+      </c>
+      <c r="E1062" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1063" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1063" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1063" t="s">
+        <v>610</v>
+      </c>
+      <c r="C1063" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1063">
+        <v>3</v>
+      </c>
+      <c r="E1063" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1064" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1064" t="s">
+        <v>465</v>
+      </c>
+      <c r="C1064" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1064">
+        <v>5</v>
+      </c>
+      <c r="E1064" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1065" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1065" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1065" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1065">
+        <v>3</v>
+      </c>
+      <c r="E1065" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1066" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1066" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1066" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1066">
+        <v>3</v>
+      </c>
+      <c r="E1066" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1067" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1067" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1067" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1067">
+        <v>2</v>
+      </c>
+      <c r="E1067" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1068" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1068" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1068" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1068">
+        <v>2</v>
+      </c>
+      <c r="E1068" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1069" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1069" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1069" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1069">
+        <v>4</v>
+      </c>
+      <c r="E1069" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1070" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1070" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1070" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1070">
+        <v>3</v>
+      </c>
+      <c r="E1070" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1071" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1071" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1071" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1071">
+        <v>2</v>
+      </c>
+      <c r="E1071" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1072" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1072" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1072" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1072">
+        <v>4</v>
+      </c>
+      <c r="E1072" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1073" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1073" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1073" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1073">
+        <v>4</v>
+      </c>
+      <c r="E1073" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1074" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1074" t="s">
+        <v>541</v>
+      </c>
+      <c r="C1074" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1074">
+        <v>2</v>
+      </c>
+      <c r="E1074" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1075" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1075" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1075" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1075" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1075">
+        <v>2</v>
+      </c>
+      <c r="E1075" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1076" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1076" t="s">
+        <v>471</v>
+      </c>
+      <c r="C1076" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1076">
+        <v>5</v>
+      </c>
+      <c r="E1076" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1077" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1077" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1077" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1077" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1077">
+        <v>1</v>
+      </c>
+      <c r="E1077" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1078" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1078" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1078" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1078">
+        <v>2</v>
+      </c>
+      <c r="E1078" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1079" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1079" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1079" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1079">
+        <v>5</v>
+      </c>
+      <c r="E1079" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1080" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1080" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1080">
+        <v>5</v>
+      </c>
+      <c r="E1080" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1081" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1081" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1081" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1081">
+        <v>2</v>
+      </c>
+      <c r="E1081" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1082" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1082" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1082" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1082">
+        <v>2</v>
+      </c>
+      <c r="E1082" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1083" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1083" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1083" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1083">
+        <v>3</v>
+      </c>
+      <c r="E1083" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1084" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1084" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1084" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1084">
+        <v>3</v>
+      </c>
+      <c r="E1084" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1085" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1085" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1085" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1085">
+        <v>5</v>
+      </c>
+      <c r="E1085" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1086" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1086" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1086" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1086">
+        <v>3</v>
+      </c>
+      <c r="E1086" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1087" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1087" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1087" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1087">
+        <v>5</v>
+      </c>
+      <c r="E1087" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1088" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1088" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1088" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1088">
+        <v>5</v>
+      </c>
+      <c r="E1088" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1089" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1089" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1089" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1089">
+        <v>5</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1090" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1090" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1090">
+        <v>2</v>
+      </c>
+      <c r="E1090" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1091" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>544</v>
+      </c>
+      <c r="C1091" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1091">
+        <v>5</v>
+      </c>
+      <c r="E1091" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1092" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1092" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1092" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1092">
+        <v>4</v>
+      </c>
+      <c r="E1092" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1093" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1093" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1093">
+        <v>2</v>
+      </c>
+      <c r="E1093" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1094" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1094" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1094" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1094">
+        <v>5</v>
+      </c>
+      <c r="E1094" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1095" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1095" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1095" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1095">
+        <v>4</v>
+      </c>
+      <c r="E1095" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1096" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1096" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1096" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1096">
+        <v>2</v>
+      </c>
+      <c r="E1096" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1097" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1097" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1097" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1097">
+        <v>5</v>
+      </c>
+      <c r="E1097" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1098" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1098" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1098" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1098">
+        <v>1</v>
+      </c>
+      <c r="E1098" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1099" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1099" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1099" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1099">
+        <v>5</v>
+      </c>
+      <c r="E1099" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1100" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1100" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1100">
+        <v>5</v>
+      </c>
+      <c r="E1100" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1101" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1101" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1101" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1101">
+        <v>5</v>
+      </c>
+      <c r="E1101" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1102" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1102" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1102" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1102">
+        <v>4</v>
+      </c>
+      <c r="E1102" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1103" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1103" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1103" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1103">
+        <v>2</v>
+      </c>
+      <c r="E1103" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1104" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1104" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1104" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1104">
+        <v>3</v>
+      </c>
+      <c r="E1104" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1105" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1105" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1105" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1105">
+        <v>5</v>
+      </c>
+      <c r="E1105" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1106" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1106" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1106" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1106">
+        <v>2</v>
+      </c>
+      <c r="E1106" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1107" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1107" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1107" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1107">
+        <v>2</v>
+      </c>
+      <c r="E1107" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1108" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1108" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1108" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1108">
+        <v>3</v>
+      </c>
+      <c r="E1108" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1109" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1109" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1109" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1109">
+        <v>2</v>
+      </c>
+      <c r="E1109" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1110" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1110" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1110" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1110">
+        <v>5</v>
+      </c>
+      <c r="E1110" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1111" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1111" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1111" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1111">
+        <v>2</v>
+      </c>
+      <c r="E1111" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1112" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1112" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1112" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1112">
+        <v>4</v>
+      </c>
+      <c r="E1112" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1113" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1113" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1113" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1113">
+        <v>3</v>
+      </c>
+      <c r="E1113" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1114" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1114" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1114" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1114">
+        <v>4</v>
+      </c>
+      <c r="E1114" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1115" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1115" t="s">
+        <v>618</v>
+      </c>
+      <c r="C1115" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1115">
+        <v>5</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1116" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1116" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1116" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1116">
+        <v>1</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1117" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1117" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1117" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1117">
+        <v>5</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1118" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1118" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1118" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1118">
+        <v>5</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1119" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1119" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1119" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1119">
+        <v>5</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1120" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1120" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1120" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1120">
+        <v>2</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1121" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1121" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1121" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1121">
+        <v>2</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1122" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1122" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1122" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1122">
+        <v>4</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1123" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1123" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1123" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1123">
+        <v>2</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1124" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1124" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1124" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1124">
+        <v>5</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1125" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1125" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1125" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1125">
+        <v>3</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1126" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1126" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1126" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1126">
+        <v>1</v>
+      </c>
+      <c r="E1126" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1127" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1127" t="s">
+        <v>158</v>
+      </c>
+      <c r="C1127" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1127">
+        <v>2</v>
+      </c>
+      <c r="E1127" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1128" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1128" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1128" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1128">
+        <v>3</v>
+      </c>
+      <c r="E1128" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1129" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1129" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1129" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1129">
+        <v>4</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1130" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1130" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1130" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1130">
+        <v>5</v>
+      </c>
+      <c r="E1130" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1131" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1131" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1131" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1131">
+        <v>3</v>
+      </c>
+      <c r="E1131" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1132" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1132" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1132" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1132">
+        <v>2</v>
+      </c>
+      <c r="E1132" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1133" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1133" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1133" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1133">
+        <v>3</v>
+      </c>
+      <c r="E1133" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1134" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1134" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1134" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1134">
+        <v>2</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1135" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1135" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1135" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1135">
+        <v>4</v>
+      </c>
+      <c r="E1135" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1136" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1136" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1136" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1136">
+        <v>1</v>
+      </c>
+      <c r="E1136" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1137" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1137" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1137" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1137">
+        <v>2</v>
+      </c>
+      <c r="E1137" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1138" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1138" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1138" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1138">
+        <v>2</v>
+      </c>
+      <c r="E1138" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1139" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1139" t="s">
+        <v>559</v>
+      </c>
+      <c r="C1139" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1139">
+        <v>3</v>
+      </c>
+      <c r="E1139" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1140" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1140" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1140" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1140" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1140">
+        <v>5</v>
+      </c>
+      <c r="E1140" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1141" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1141" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1141" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1141">
+        <v>5</v>
+      </c>
+      <c r="E1141" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1142" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1142" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1142" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1142">
+        <v>2</v>
+      </c>
+      <c r="E1142" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1143" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1143" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1143" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1143">
+        <v>3</v>
+      </c>
+      <c r="E1143" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1144" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1144" t="s">
+        <v>560</v>
+      </c>
+      <c r="C1144" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1144">
+        <v>3</v>
+      </c>
+      <c r="E1144" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1145" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1145" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1145" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1145">
+        <v>3</v>
+      </c>
+      <c r="E1145" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1146" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1146" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1146" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1146">
+        <v>4</v>
+      </c>
+      <c r="E1146" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1147" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1147" t="s">
+        <v>184</v>
+      </c>
+      <c r="C1147" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1147">
+        <v>3</v>
+      </c>
+      <c r="E1147" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1148" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1148" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1148" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1148">
+        <v>2</v>
+      </c>
+      <c r="E1148" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1149" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1149" t="s">
+        <v>625</v>
+      </c>
+      <c r="C1149" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1149">
+        <v>3</v>
+      </c>
+      <c r="E1149" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1150" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1150" t="s">
+        <v>626</v>
+      </c>
+      <c r="C1150" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1150">
+        <v>3</v>
+      </c>
+      <c r="E1150" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1151" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1151" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1151" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1151">
+        <v>4</v>
+      </c>
+      <c r="E1151" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1152" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1152" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1152" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1152">
+        <v>4</v>
+      </c>
+      <c r="E1152" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1153" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1153" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1153" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1153">
+        <v>2</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1154" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1154" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1154" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1154">
+        <v>3</v>
+      </c>
+      <c r="E1154" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1155" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1155" t="s">
+        <v>194</v>
+      </c>
+      <c r="C1155" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1155">
+        <v>2</v>
+      </c>
+      <c r="E1155" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1156" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1156" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1156" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1156">
+        <v>4</v>
+      </c>
+      <c r="E1156" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1157" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1157" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1157" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1157">
+        <v>5</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1158" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1158" t="s">
+        <v>198</v>
+      </c>
+      <c r="C1158" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1158">
+        <v>1</v>
+      </c>
+      <c r="E1158" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1159" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1159" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1159" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1159">
+        <v>5</v>
+      </c>
+      <c r="E1159" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1160" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1160" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1160" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1160">
+        <v>2</v>
+      </c>
+      <c r="E1160" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1161" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1161" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1161" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1161">
+        <v>2</v>
+      </c>
+      <c r="E1161" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1162" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1162" t="s">
+        <v>207</v>
+      </c>
+      <c r="C1162" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1162">
+        <v>1</v>
+      </c>
+      <c r="E1162" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1163" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1163" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1163" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1163">
+        <v>4</v>
+      </c>
+      <c r="E1163" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1164" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1164" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1164" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1164">
+        <v>5</v>
+      </c>
+      <c r="E1164" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1165" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1165" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1165" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1165">
+        <v>1</v>
+      </c>
+      <c r="E1165" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1166" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1166" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1166" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1166">
+        <v>2</v>
+      </c>
+      <c r="E1166" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1167" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1167" t="s">
+        <v>215</v>
+      </c>
+      <c r="C1167" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1167">
+        <v>3</v>
+      </c>
+      <c r="E1167" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1168" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1168" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1168" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1168">
+        <v>3</v>
+      </c>
+      <c r="E1168" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1169" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1169" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1169" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1169">
+        <v>4</v>
+      </c>
+      <c r="E1169" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1170" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1170" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1170" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1170">
+        <v>2</v>
+      </c>
+      <c r="E1170" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1171" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1171" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1171" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1171">
+        <v>5</v>
+      </c>
+      <c r="E1171" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1172" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1172" t="s">
+        <v>223</v>
+      </c>
+      <c r="C1172" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1172">
+        <v>2</v>
+      </c>
+      <c r="E1172" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1173" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1173" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1173" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1173">
+        <v>4</v>
+      </c>
+      <c r="E1173" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1174" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1174" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1174" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1174">
+        <v>1</v>
+      </c>
+      <c r="E1174" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1175" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1175" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1175" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1175">
+        <v>2</v>
+      </c>
+      <c r="E1175" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1176" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1176" t="s">
+        <v>231</v>
+      </c>
+      <c r="C1176" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1176">
+        <v>5</v>
+      </c>
+      <c r="E1176" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1177" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1177" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1177" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1177">
+        <v>1</v>
+      </c>
+      <c r="E1177" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1178" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1178" t="s">
+        <v>633</v>
+      </c>
+      <c r="C1178" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1178">
+        <v>2</v>
+      </c>
+      <c r="E1178" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1179" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1179" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1179" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1179">
+        <v>3</v>
+      </c>
+      <c r="E1179" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1180" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1180" t="s">
+        <v>577</v>
+      </c>
+      <c r="C1180" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1180">
+        <v>5</v>
+      </c>
+      <c r="E1180" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1181" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1181" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1181" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1181">
+        <v>2</v>
+      </c>
+      <c r="E1181" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1182" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1182" t="s">
+        <v>634</v>
+      </c>
+      <c r="C1182" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1182">
+        <v>2</v>
+      </c>
+      <c r="E1182" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1183" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1183" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1183" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1183">
+        <v>2</v>
+      </c>
+      <c r="E1183" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1184" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1184" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1184" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1184">
+        <v>5</v>
+      </c>
+      <c r="E1184" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1185" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1185" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1185" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1185">
+        <v>2</v>
+      </c>
+      <c r="E1185" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1186" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1186" t="s">
+        <v>239</v>
+      </c>
+      <c r="C1186" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1186">
+        <v>3</v>
+      </c>
+      <c r="E1186" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1187" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1187" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1187" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1187">
+        <v>2</v>
+      </c>
+      <c r="E1187" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1188" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1188" t="s">
+        <v>242</v>
+      </c>
+      <c r="C1188" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1188">
+        <v>5</v>
+      </c>
+      <c r="E1188" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1189" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1189" t="s">
+        <v>636</v>
+      </c>
+      <c r="C1189" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1189">
+        <v>2</v>
+      </c>
+      <c r="E1189" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1190" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1190" t="s">
+        <v>637</v>
+      </c>
+      <c r="C1190" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1190">
+        <v>3</v>
+      </c>
+      <c r="E1190" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1191" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1191" t="s">
+        <v>244</v>
+      </c>
+      <c r="C1191" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1191">
+        <v>2</v>
+      </c>
+      <c r="E1191" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1192" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1192" t="s">
+        <v>247</v>
+      </c>
+      <c r="C1192" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1192">
+        <v>5</v>
+      </c>
+      <c r="E1192" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1193" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1193" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1193" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1193">
+        <v>5</v>
+      </c>
+      <c r="E1193" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1194" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1194" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1194" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1194">
+        <v>5</v>
+      </c>
+      <c r="E1194" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1195" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1195" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1195" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1195">
+        <v>3</v>
+      </c>
+      <c r="E1195" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1196" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1196" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1196" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1196">
+        <v>1</v>
+      </c>
+      <c r="E1196" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1197" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>640</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1197">
+        <v>3</v>
+      </c>
+      <c r="E1197" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1198" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>641</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1198">
+        <v>3</v>
+      </c>
+      <c r="E1198" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1199" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>255</v>
+      </c>
+      <c r="C1199" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1199">
+        <v>2</v>
+      </c>
+      <c r="E1199" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1200" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1200" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1200" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1200">
+        <v>3</v>
+      </c>
+      <c r="E1200" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1201" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1201" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1201" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1201">
+        <v>3</v>
+      </c>
+      <c r="E1201" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1202" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1202" t="s">
+        <v>585</v>
+      </c>
+      <c r="C1202" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1202">
+        <v>3</v>
+      </c>
+      <c r="E1202" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1203" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1203" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1203" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1203">
+        <v>2</v>
+      </c>
+      <c r="E1203" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1204" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1204" t="s">
+        <v>261</v>
+      </c>
+      <c r="C1204" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1204">
+        <v>3</v>
+      </c>
+      <c r="E1204" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1205" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1205" t="s">
+        <v>262</v>
+      </c>
+      <c r="C1205" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1205">
+        <v>5</v>
+      </c>
+      <c r="E1205" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1206" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1206" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1206" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1206">
+        <v>5</v>
+      </c>
+      <c r="E1206" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1207" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1207" t="s">
+        <v>264</v>
+      </c>
+      <c r="C1207" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1207">
+        <v>2</v>
+      </c>
+      <c r="E1207" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1208" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1208" t="s">
+        <v>643</v>
+      </c>
+      <c r="C1208" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1208">
+        <v>3</v>
+      </c>
+      <c r="E1208" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1209" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1209" t="s">
+        <v>644</v>
+      </c>
+      <c r="C1209" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1209">
+        <v>3</v>
+      </c>
+      <c r="E1209" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1210" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1210" t="s">
+        <v>267</v>
+      </c>
+      <c r="C1210" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1210">
+        <v>5</v>
+      </c>
+      <c r="E1210" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1211" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1211" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1211" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1211">
+        <v>1</v>
+      </c>
+      <c r="E1211" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1212" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1212" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1212" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1212">
+        <v>5</v>
+      </c>
+      <c r="E1212" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1213" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1213" t="s">
+        <v>271</v>
+      </c>
+      <c r="C1213" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1213">
+        <v>3</v>
+      </c>
+      <c r="E1213" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1214" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1214" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1214" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1214">
+        <v>3</v>
+      </c>
+      <c r="E1214" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1215" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1215" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1215" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1215">
+        <v>2</v>
+      </c>
+      <c r="E1215" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1216" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1216" t="s">
+        <v>645</v>
+      </c>
+      <c r="C1216" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1216">
+        <v>2</v>
+      </c>
+      <c r="E1216" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1217" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1217" t="s">
+        <v>274</v>
+      </c>
+      <c r="C1217" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1217">
+        <v>5</v>
+      </c>
+      <c r="E1217" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="1218" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1218" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1218" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1218" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1218">
+        <v>4</v>
+      </c>
+      <c r="E1218" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="1219" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1219" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1219" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1219" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1219">
+        <v>5</v>
+      </c>
+      <c r="E1219" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1220" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1220" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1220" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1220">
+        <v>2</v>
+      </c>
+      <c r="E1220" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1221" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1221" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1221" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1221">
+        <v>4</v>
+      </c>
+      <c r="E1221" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1222" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1222" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1222" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1222">
+        <v>5</v>
+      </c>
+      <c r="E1222" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1223" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1223" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1223" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1223">
+        <v>2</v>
+      </c>
+      <c r="E1223" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1224" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1224" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1224" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1224" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1224">
+        <v>5</v>
+      </c>
+      <c r="E1224" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1225" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1225" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1225" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1225">
+        <v>5</v>
+      </c>
+      <c r="E1225" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1226" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1226" t="s">
+        <v>282</v>
+      </c>
+      <c r="C1226" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1226">
+        <v>3</v>
+      </c>
+      <c r="E1226" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="1227" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1227" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1227" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1227" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1227">
+        <v>3</v>
+      </c>
+      <c r="E1227" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1228" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1228" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1228" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1228">
+        <v>5</v>
+      </c>
+      <c r="E1228" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1229" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1229" t="s">
+        <v>285</v>
+      </c>
+      <c r="C1229" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1229">
+        <v>5</v>
+      </c>
+      <c r="E1229" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="1230" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1230" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1230" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1230" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1230">
+        <v>1</v>
+      </c>
+      <c r="E1230" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1231" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1231" t="s">
+        <v>649</v>
+      </c>
+      <c r="C1231" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1231">
+        <v>3</v>
+      </c>
+      <c r="E1231" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1232" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1232" t="s">
+        <v>650</v>
+      </c>
+      <c r="C1232" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1232">
+        <v>3</v>
+      </c>
+      <c r="E1232" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="1233" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1233" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1233" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1233" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1233">
+        <v>2</v>
+      </c>
+      <c r="E1233" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1234" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1234" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1234" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1234">
+        <v>2</v>
+      </c>
+      <c r="E1234" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1235" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1235" t="s">
+        <v>652</v>
+      </c>
+      <c r="C1235" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1235">
+        <v>3</v>
+      </c>
+      <c r="E1235" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1236" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1236" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1236" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1236" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1236">
+        <v>4</v>
+      </c>
+      <c r="E1236" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="1237" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1237" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1237" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1237" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1237">
+        <v>5</v>
+      </c>
+      <c r="E1237" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="1238" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1238" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1238" t="s">
+        <v>294</v>
+      </c>
+      <c r="C1238" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1238">
+        <v>2</v>
+      </c>
+      <c r="E1238" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="1239" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1239" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1239" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1239" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1239">
+        <v>3</v>
+      </c>
+      <c r="E1239" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1240" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1240" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1240" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1240" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1240">
+        <v>3</v>
+      </c>
+      <c r="E1240" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1241" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1241" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1241" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1241" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1241">
+        <v>4</v>
+      </c>
+      <c r="E1241" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1242" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1242" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1242" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1242">
+        <v>3</v>
+      </c>
+      <c r="E1242" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1243" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1243" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1243" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1243">
+        <v>5</v>
+      </c>
+      <c r="E1243" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1244" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1244" t="s">
+        <v>302</v>
+      </c>
+      <c r="C1244" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1244">
+        <v>3</v>
+      </c>
+      <c r="E1244" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1245" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1245" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1245" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1245">
+        <v>3</v>
+      </c>
+      <c r="E1245" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1246" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1246" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1246" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1246">
+        <v>2</v>
+      </c>
+      <c r="E1246" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1247" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1247" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1247" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1247">
+        <v>2</v>
+      </c>
+      <c r="E1247" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1248" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1248" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1248" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1248">
+        <v>3</v>
+      </c>
+      <c r="E1248" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="1249" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1249" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1249" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1249" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1249">
+        <v>1</v>
+      </c>
+      <c r="E1249" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1250" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1250" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B1250" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1250" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1250">
+        <v>3</v>
+      </c>
+      <c r="E1250" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
home page: add new data announcement banner + concern group movement cards
</commit_message>
<xml_diff>
--- a/Tutor_Concerns.xlsx
+++ b/Tutor_Concerns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tylerharrington/Desktop/Revolution Prep/FL_Dashboards/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FB3B8C77-89FE-B043-91B9-CEBE9FB282DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B7E57B33-0637-4E4B-971B-1977EBD743D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{92DEE1D6-509C-344A-AA8F-D8DD2317BD81}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17860" xr2:uid="{92DEE1D6-509C-344A-AA8F-D8DD2317BD81}"/>
   </bookViews>
   <sheets>
     <sheet name="Concerns" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5909" uniqueCount="705">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="6833" uniqueCount="744">
   <si>
     <t>Tutor Name</t>
   </si>
@@ -2151,6 +2151,123 @@
   </si>
   <si>
     <t>1/25/26 - 2/21/26</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % Sessions on Time &lt; 90%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Anna Jasko</t>
+  </si>
+  <si>
+    <t>Brian Johnson</t>
+  </si>
+  <si>
+    <t>Cadence Liles</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Craig Street</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Debleena Chatterjee</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Weighted Repurchases = 0</t>
+  </si>
+  <si>
+    <t>Guha Sriram</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>John Salcedo</t>
+  </si>
+  <si>
+    <t>Justin Hill</t>
+  </si>
+  <si>
+    <t>Kate Haldeman</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Weighted Repurchases = 0</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>Nisha Fletcher</t>
+  </si>
+  <si>
+    <t>Parthav Elangovan</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % Sessions on Time &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 90%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Weighted Repurchases = 0; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Vincent Cross</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Weighted Repurchases = 0; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>2/22/26 - 3/21/26</t>
   </si>
 </sst>
 </file>
@@ -3020,7 +3137,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA4CB91-83C8-694D-BBCD-170E9881DA10}">
-  <dimension ref="A1:E1477"/>
+  <dimension ref="A1:E1708"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -28135,6 +28252,3933 @@
         <v>703</v>
       </c>
     </row>
+    <row r="1478" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1478" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1478" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1478" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1478">
+        <v>2</v>
+      </c>
+      <c r="E1478" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1479" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1479" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1479" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1479" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1479">
+        <v>2</v>
+      </c>
+      <c r="E1479" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1480" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1480" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1480" t="s">
+        <v>657</v>
+      </c>
+      <c r="C1480" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1480">
+        <v>5</v>
+      </c>
+      <c r="E1480" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="1481" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1481" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1481" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1481" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1481">
+        <v>4</v>
+      </c>
+      <c r="E1481" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="1482" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1482" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1482" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1482" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1482">
+        <v>1</v>
+      </c>
+      <c r="E1482" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1483" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1483" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1483" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1483" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1483">
+        <v>1</v>
+      </c>
+      <c r="E1483" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1484" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1484" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1484" t="s">
+        <v>659</v>
+      </c>
+      <c r="C1484" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1484">
+        <v>5</v>
+      </c>
+      <c r="E1484" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="1485" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1485" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1485" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1485" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1485">
+        <v>3</v>
+      </c>
+      <c r="E1485" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="1486" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1486" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1486" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1486" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1486">
+        <v>2</v>
+      </c>
+      <c r="E1486" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="1487" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1487" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1487" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1487" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1487">
+        <v>4</v>
+      </c>
+      <c r="E1487" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1488" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1488" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1488" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1488" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1488">
+        <v>5</v>
+      </c>
+      <c r="E1488" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1489" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1489" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1489" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1489">
+        <v>5</v>
+      </c>
+      <c r="E1489" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1490" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1490" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1490" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1490">
+        <v>5</v>
+      </c>
+      <c r="E1490" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1491" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1491" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1491" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1491">
+        <v>3</v>
+      </c>
+      <c r="E1491" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1492" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1492" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1492" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1492">
+        <v>5</v>
+      </c>
+      <c r="E1492" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1493" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1493" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1493" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1493">
+        <v>4</v>
+      </c>
+      <c r="E1493" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1494" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1494" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1494" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1494">
+        <v>5</v>
+      </c>
+      <c r="E1494" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1495" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1495" t="s">
+        <v>663</v>
+      </c>
+      <c r="C1495" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1495">
+        <v>5</v>
+      </c>
+      <c r="E1495" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1496" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1496" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1496" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1496">
+        <v>2</v>
+      </c>
+      <c r="E1496" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1497" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1497" t="s">
+        <v>709</v>
+      </c>
+      <c r="C1497" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1497">
+        <v>3</v>
+      </c>
+      <c r="E1497" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1498" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1498" t="s">
+        <v>607</v>
+      </c>
+      <c r="C1498" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1498">
+        <v>5</v>
+      </c>
+      <c r="E1498" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1499" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1499" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1499" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1499" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1499">
+        <v>1</v>
+      </c>
+      <c r="E1499" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1500" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1500" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1500" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1500">
+        <v>2</v>
+      </c>
+      <c r="E1500" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1501" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1501" t="s">
+        <v>534</v>
+      </c>
+      <c r="C1501" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1501">
+        <v>5</v>
+      </c>
+      <c r="E1501" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1502" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1502" t="s">
+        <v>665</v>
+      </c>
+      <c r="C1502" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1502">
+        <v>3</v>
+      </c>
+      <c r="E1502" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1503" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1503" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1503" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1503">
+        <v>4</v>
+      </c>
+      <c r="E1503" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="1504" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1504" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1504" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1504" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1504">
+        <v>2</v>
+      </c>
+      <c r="E1504" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1505" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1505" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1505" t="s">
+        <v>609</v>
+      </c>
+      <c r="C1505" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1505">
+        <v>5</v>
+      </c>
+      <c r="E1505" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1506" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1506" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1506" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1506" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1506">
+        <v>2</v>
+      </c>
+      <c r="E1506" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1507" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1507" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1507" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1507" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1507">
+        <v>2</v>
+      </c>
+      <c r="E1507" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1508" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1508" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1508" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1508" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1508">
+        <v>2</v>
+      </c>
+      <c r="E1508" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1509" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1509" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1509" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1509" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1509">
+        <v>2</v>
+      </c>
+      <c r="E1509" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1510" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1510" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1510" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1510" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1510">
+        <v>5</v>
+      </c>
+      <c r="E1510" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1511" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1511" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1511" t="s">
+        <v>710</v>
+      </c>
+      <c r="C1511" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1511">
+        <v>5</v>
+      </c>
+      <c r="E1511" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="1512" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1512" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1512" t="s">
+        <v>610</v>
+      </c>
+      <c r="C1512" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1512">
+        <v>4</v>
+      </c>
+      <c r="E1512" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1513" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1513" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1513" t="s">
+        <v>465</v>
+      </c>
+      <c r="C1513" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1513">
+        <v>2</v>
+      </c>
+      <c r="E1513" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1514" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1514" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1514" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1514" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1514">
+        <v>2</v>
+      </c>
+      <c r="E1514" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1515" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1515" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1515" t="s">
+        <v>711</v>
+      </c>
+      <c r="C1515" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1515">
+        <v>3</v>
+      </c>
+      <c r="E1515" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1516" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1516" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1516" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1516" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1516">
+        <v>5</v>
+      </c>
+      <c r="E1516" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="1517" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1517" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1517" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1517" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1517">
+        <v>5</v>
+      </c>
+      <c r="E1517" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1518" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1518" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1518" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1518" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1518">
+        <v>1</v>
+      </c>
+      <c r="E1518" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1519" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1519" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1519" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1519" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1519">
+        <v>4</v>
+      </c>
+      <c r="E1519" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1520" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1520" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1520" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1520">
+        <v>4</v>
+      </c>
+      <c r="E1520" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1521" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1521" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1521" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1521">
+        <v>1</v>
+      </c>
+      <c r="E1521" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1522" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1522" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1522" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1522">
+        <v>1</v>
+      </c>
+      <c r="E1522" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1523" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1523" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1523" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1523" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1523">
+        <v>2</v>
+      </c>
+      <c r="E1523" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1524" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1524" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1524" t="s">
+        <v>668</v>
+      </c>
+      <c r="C1524" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1524">
+        <v>4</v>
+      </c>
+      <c r="E1524" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="1525" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1525" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1525" t="s">
+        <v>541</v>
+      </c>
+      <c r="C1525" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1525">
+        <v>1</v>
+      </c>
+      <c r="E1525" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1526" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1526" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1526" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1526" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1526">
+        <v>2</v>
+      </c>
+      <c r="E1526" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1527" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1527" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1527" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1527" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1527">
+        <v>3</v>
+      </c>
+      <c r="E1527" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="1528" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1528" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1528" t="s">
+        <v>471</v>
+      </c>
+      <c r="C1528" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1528">
+        <v>3</v>
+      </c>
+      <c r="E1528" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1529" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1529" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1529" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1529" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1529">
+        <v>1</v>
+      </c>
+      <c r="E1529" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1530" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1530" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1530" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1530" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1530">
+        <v>2</v>
+      </c>
+      <c r="E1530" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1531" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1531" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1531" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1531" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1531">
+        <v>2</v>
+      </c>
+      <c r="E1531" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1532" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1532" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1532" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1532" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1532">
+        <v>2</v>
+      </c>
+      <c r="E1532" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1533" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1533" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1533" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1533" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1533">
+        <v>2</v>
+      </c>
+      <c r="E1533" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1534" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1534" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1534" t="s">
+        <v>713</v>
+      </c>
+      <c r="C1534" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1534">
+        <v>5</v>
+      </c>
+      <c r="E1534" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="1535" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1535" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1535" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1535" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1535">
+        <v>2</v>
+      </c>
+      <c r="E1535" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1536" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1536" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1536" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1536" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1536">
+        <v>4</v>
+      </c>
+      <c r="E1536" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="1537" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1537" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1537" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1537" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1537">
+        <v>5</v>
+      </c>
+      <c r="E1537" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1538" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1538" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1538" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1538" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1538">
+        <v>2</v>
+      </c>
+      <c r="E1538" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1539" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1539" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1539" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1539" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1539">
+        <v>4</v>
+      </c>
+      <c r="E1539" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="1540" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1540" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1540" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1540" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1540">
+        <v>1</v>
+      </c>
+      <c r="E1540" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1541" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1541" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1541" t="s">
+        <v>716</v>
+      </c>
+      <c r="C1541" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1541">
+        <v>2</v>
+      </c>
+      <c r="E1541" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1542" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1542" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1542" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1542" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1542">
+        <v>5</v>
+      </c>
+      <c r="E1542" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="1543" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1543" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1543" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1543" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1543">
+        <v>2</v>
+      </c>
+      <c r="E1543" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1544" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1544" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1544" t="s">
+        <v>544</v>
+      </c>
+      <c r="C1544" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1544">
+        <v>5</v>
+      </c>
+      <c r="E1544" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="1545" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1545" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1545" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1545" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1545">
+        <v>5</v>
+      </c>
+      <c r="E1545" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="1546" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1546" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1546" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1546" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1546">
+        <v>2</v>
+      </c>
+      <c r="E1546" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1547" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1547" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1547" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1547" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1547">
+        <v>3</v>
+      </c>
+      <c r="E1547" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1548" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1548" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1548" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1548" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1548">
+        <v>3</v>
+      </c>
+      <c r="E1548" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1549" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1549" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1549" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1549">
+        <v>2</v>
+      </c>
+      <c r="E1549" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1550" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1550" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1550" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1550">
+        <v>5</v>
+      </c>
+      <c r="E1550" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="1551" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1551" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1551" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1551" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1551">
+        <v>2</v>
+      </c>
+      <c r="E1551" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="1552" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1552" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1552" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1552" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1552">
+        <v>2</v>
+      </c>
+      <c r="E1552" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="1553" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1553" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1553" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1553" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1553">
+        <v>5</v>
+      </c>
+      <c r="E1553" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1554" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1554" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1554" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1554" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1554">
+        <v>4</v>
+      </c>
+      <c r="E1554" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1555" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1555" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1555" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1555" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1555">
+        <v>5</v>
+      </c>
+      <c r="E1555" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="1556" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1556" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1556" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1556" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1556">
+        <v>4</v>
+      </c>
+      <c r="E1556" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="1557" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1557" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1557" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1557" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1557">
+        <v>5</v>
+      </c>
+      <c r="E1557" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="1558" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1558" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1558" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1558" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1558">
+        <v>2</v>
+      </c>
+      <c r="E1558" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1559" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1559" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1559" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1559" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1559">
+        <v>2</v>
+      </c>
+      <c r="E1559" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1560" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1560" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1560" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1560" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1560">
+        <v>2</v>
+      </c>
+      <c r="E1560" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1561" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1561" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1561" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1561" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1561">
+        <v>2</v>
+      </c>
+      <c r="E1561" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1562" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1562" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1562" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1562" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1562">
+        <v>4</v>
+      </c>
+      <c r="E1562" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1563" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1563" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1563" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1563">
+        <v>3</v>
+      </c>
+      <c r="E1563" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1564" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1564" t="s">
+        <v>720</v>
+      </c>
+      <c r="C1564" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1564">
+        <v>3</v>
+      </c>
+      <c r="E1564" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1565" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1565" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1565" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1565">
+        <v>2</v>
+      </c>
+      <c r="E1565" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1566" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1566" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1566" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1566">
+        <v>3</v>
+      </c>
+      <c r="E1566" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1567" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1567" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1567" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1567">
+        <v>4</v>
+      </c>
+      <c r="E1567" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1568" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1568" t="s">
+        <v>673</v>
+      </c>
+      <c r="C1568" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1568">
+        <v>5</v>
+      </c>
+      <c r="E1568" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1569" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1569" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1569" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1569">
+        <v>2</v>
+      </c>
+      <c r="E1569" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1570" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1570" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1570" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1570">
+        <v>4</v>
+      </c>
+      <c r="E1570" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1571" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1571" t="s">
+        <v>675</v>
+      </c>
+      <c r="C1571" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1571">
+        <v>3</v>
+      </c>
+      <c r="E1571" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1572" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1572" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1572" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1572">
+        <v>5</v>
+      </c>
+      <c r="E1572" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1573" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1573" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1573" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1573">
+        <v>5</v>
+      </c>
+      <c r="E1573" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1574" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1574" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1574" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1574">
+        <v>2</v>
+      </c>
+      <c r="E1574" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1575" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1575" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1575" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1575">
+        <v>2</v>
+      </c>
+      <c r="E1575" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1576" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1576" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1576" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1576">
+        <v>1</v>
+      </c>
+      <c r="E1576" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1577" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1577" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1577" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1577">
+        <v>4</v>
+      </c>
+      <c r="E1577" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1578" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1578" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1578" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1578">
+        <v>5</v>
+      </c>
+      <c r="E1578" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1579" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1579" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1579" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1579">
+        <v>2</v>
+      </c>
+      <c r="E1579" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1580" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1580" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1580" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1580">
+        <v>2</v>
+      </c>
+      <c r="E1580" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1581" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1581" t="s">
+        <v>158</v>
+      </c>
+      <c r="C1581" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1581">
+        <v>2</v>
+      </c>
+      <c r="E1581" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1582" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1582" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1582" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1582">
+        <v>2</v>
+      </c>
+      <c r="E1582" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1583" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1583" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1583" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1583">
+        <v>2</v>
+      </c>
+      <c r="E1583" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1584" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1584" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1584" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1584">
+        <v>2</v>
+      </c>
+      <c r="E1584" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1585" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1585" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1585" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1585">
+        <v>2</v>
+      </c>
+      <c r="E1585" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1586" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1586" t="s">
+        <v>678</v>
+      </c>
+      <c r="C1586" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1586">
+        <v>5</v>
+      </c>
+      <c r="E1586" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1587" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1587" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1587" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1587">
+        <v>2</v>
+      </c>
+      <c r="E1587" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1588" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1588" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1588" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1588" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1588">
+        <v>3</v>
+      </c>
+      <c r="E1588" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1589" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1589" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1589" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1589">
+        <v>2</v>
+      </c>
+      <c r="E1589" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1590" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1590" t="s">
+        <v>722</v>
+      </c>
+      <c r="C1590" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1590">
+        <v>3</v>
+      </c>
+      <c r="E1590" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1591" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1591" t="s">
+        <v>680</v>
+      </c>
+      <c r="C1591" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1591">
+        <v>2</v>
+      </c>
+      <c r="E1591" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1592" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1592" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1592" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1592">
+        <v>3</v>
+      </c>
+      <c r="E1592" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1593" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1593" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1593" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1593">
+        <v>2</v>
+      </c>
+      <c r="E1593" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1594" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1594" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1594" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1594">
+        <v>4</v>
+      </c>
+      <c r="E1594" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1595" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1595" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1595" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1595">
+        <v>2</v>
+      </c>
+      <c r="E1595" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1596" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1596" t="s">
+        <v>559</v>
+      </c>
+      <c r="C1596" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1596">
+        <v>1</v>
+      </c>
+      <c r="E1596" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1597" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1597" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1597" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1597">
+        <v>2</v>
+      </c>
+      <c r="E1597" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1598" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1598" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1598" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1598">
+        <v>5</v>
+      </c>
+      <c r="E1598" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1599" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1599" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1599" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1599">
+        <v>1</v>
+      </c>
+      <c r="E1599" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1600" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1600" t="s">
+        <v>723</v>
+      </c>
+      <c r="C1600" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1600">
+        <v>3</v>
+      </c>
+      <c r="E1600" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1601" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1601" t="s">
+        <v>682</v>
+      </c>
+      <c r="C1601" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1601">
+        <v>5</v>
+      </c>
+      <c r="E1601" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1602" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1602" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1602" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1602">
+        <v>3</v>
+      </c>
+      <c r="E1602" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1603" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1603" t="s">
+        <v>560</v>
+      </c>
+      <c r="C1603" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1603">
+        <v>2</v>
+      </c>
+      <c r="E1603" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1604" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1604" t="s">
+        <v>724</v>
+      </c>
+      <c r="C1604" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1604">
+        <v>3</v>
+      </c>
+      <c r="E1604" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1605" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1605" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1605" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1605">
+        <v>5</v>
+      </c>
+      <c r="E1605" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1606" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1606" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1606" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1606">
+        <v>5</v>
+      </c>
+      <c r="E1606" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1607" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1607" t="s">
+        <v>184</v>
+      </c>
+      <c r="C1607" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1607">
+        <v>3</v>
+      </c>
+      <c r="E1607" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1608" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1608" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1608" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1608">
+        <v>2</v>
+      </c>
+      <c r="E1608" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1609" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1609" t="s">
+        <v>626</v>
+      </c>
+      <c r="C1609" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1609">
+        <v>5</v>
+      </c>
+      <c r="E1609" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1610" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1610" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1610" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1610">
+        <v>5</v>
+      </c>
+      <c r="E1610" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1611" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1611" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1611" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1611">
+        <v>5</v>
+      </c>
+      <c r="E1611" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1612" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1612" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1612" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1612">
+        <v>5</v>
+      </c>
+      <c r="E1612" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1613" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1613" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1613" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1613">
+        <v>5</v>
+      </c>
+      <c r="E1613" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1614" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1614" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1614" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1614">
+        <v>5</v>
+      </c>
+      <c r="E1614" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1615" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1615" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1615" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1615">
+        <v>1</v>
+      </c>
+      <c r="E1615" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1616" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1616" t="s">
+        <v>198</v>
+      </c>
+      <c r="C1616" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1616">
+        <v>1</v>
+      </c>
+      <c r="E1616" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1617" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1617" t="s">
+        <v>685</v>
+      </c>
+      <c r="C1617" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1617">
+        <v>5</v>
+      </c>
+      <c r="E1617" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="1618" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1618" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1618" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1618" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1618">
+        <v>3</v>
+      </c>
+      <c r="E1618" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1619" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1619" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1619" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1619" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1619">
+        <v>3</v>
+      </c>
+      <c r="E1619" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1620" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1620" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1620" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1620" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1620">
+        <v>2</v>
+      </c>
+      <c r="E1620" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1621" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1621" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1621" t="s">
+        <v>207</v>
+      </c>
+      <c r="C1621" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1621">
+        <v>2</v>
+      </c>
+      <c r="E1621" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1622" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1622" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1622" t="s">
+        <v>686</v>
+      </c>
+      <c r="C1622" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1622">
+        <v>5</v>
+      </c>
+      <c r="E1622" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="1623" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1623" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1623" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1623" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1623">
+        <v>2</v>
+      </c>
+      <c r="E1623" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1624" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1624" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1624" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1624" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1624">
+        <v>2</v>
+      </c>
+      <c r="E1624" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1625" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1625" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1625" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1625" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1625">
+        <v>2</v>
+      </c>
+      <c r="E1625" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1626" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1626" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1626" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1626" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1626">
+        <v>3</v>
+      </c>
+      <c r="E1626" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1627" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1627" t="s">
+        <v>215</v>
+      </c>
+      <c r="C1627" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1627">
+        <v>5</v>
+      </c>
+      <c r="E1627" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1628" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1628" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1628" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1628" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1628">
+        <v>5</v>
+      </c>
+      <c r="E1628" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1629" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1629" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1629" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1629">
+        <v>5</v>
+      </c>
+      <c r="E1629" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1630" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1630" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1630" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1630" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1630">
+        <v>2</v>
+      </c>
+      <c r="E1630" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1631" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1631" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1631" t="s">
+        <v>691</v>
+      </c>
+      <c r="C1631" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1631">
+        <v>2</v>
+      </c>
+      <c r="E1631" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1632" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1632" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1632" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1632" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1632">
+        <v>2</v>
+      </c>
+      <c r="E1632" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1633" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1633" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1633" t="s">
+        <v>223</v>
+      </c>
+      <c r="C1633" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1633">
+        <v>3</v>
+      </c>
+      <c r="E1633" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="1634" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1634" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1634" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1634" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1634">
+        <v>2</v>
+      </c>
+      <c r="E1634" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1635" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1635" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1635" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1635" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1635">
+        <v>2</v>
+      </c>
+      <c r="E1635" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1636" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1636" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1636" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1636">
+        <v>4</v>
+      </c>
+      <c r="E1636" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1637" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1637" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1637" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1637">
+        <v>1</v>
+      </c>
+      <c r="E1637" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1638" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1638" t="s">
+        <v>633</v>
+      </c>
+      <c r="C1638" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1638">
+        <v>5</v>
+      </c>
+      <c r="E1638" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1639" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1639" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1639" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1639">
+        <v>2</v>
+      </c>
+      <c r="E1639" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1640" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1640" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1640" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1640">
+        <v>1</v>
+      </c>
+      <c r="E1640" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1641" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1641" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1641" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1641">
+        <v>2</v>
+      </c>
+      <c r="E1641" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1642" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1642" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1642" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1642">
+        <v>4</v>
+      </c>
+      <c r="E1642" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1643" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1643" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1643" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1643">
+        <v>2</v>
+      </c>
+      <c r="E1643" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1644" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1644" t="s">
+        <v>239</v>
+      </c>
+      <c r="C1644" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1644">
+        <v>5</v>
+      </c>
+      <c r="E1644" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1645" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1645" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1645" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1645">
+        <v>2</v>
+      </c>
+      <c r="E1645" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1646" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1646" t="s">
+        <v>242</v>
+      </c>
+      <c r="C1646" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1646">
+        <v>3</v>
+      </c>
+      <c r="E1646" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1647" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1647" t="s">
+        <v>729</v>
+      </c>
+      <c r="C1647" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1647">
+        <v>2</v>
+      </c>
+      <c r="E1647" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1648" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1648" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1648" t="s">
+        <v>636</v>
+      </c>
+      <c r="C1648" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1648">
+        <v>5</v>
+      </c>
+      <c r="E1648" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1649" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1649" t="s">
+        <v>637</v>
+      </c>
+      <c r="C1649" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1649">
+        <v>4</v>
+      </c>
+      <c r="E1649" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1650" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1650" t="s">
+        <v>730</v>
+      </c>
+      <c r="C1650" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1650">
+        <v>3</v>
+      </c>
+      <c r="E1650" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1651" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1651" t="s">
+        <v>244</v>
+      </c>
+      <c r="C1651" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1651">
+        <v>5</v>
+      </c>
+      <c r="E1651" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1652" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1652" t="s">
+        <v>247</v>
+      </c>
+      <c r="C1652" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1652">
+        <v>5</v>
+      </c>
+      <c r="E1652" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1653" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1653" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1653" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1653">
+        <v>5</v>
+      </c>
+      <c r="E1653" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1654" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1654" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1654" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1654">
+        <v>3</v>
+      </c>
+      <c r="E1654" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1655" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1655" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1655" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1655">
+        <v>3</v>
+      </c>
+      <c r="E1655" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1656" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1656" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1656" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1656">
+        <v>5</v>
+      </c>
+      <c r="E1656" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1657" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1657" t="s">
+        <v>640</v>
+      </c>
+      <c r="C1657" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1657">
+        <v>5</v>
+      </c>
+      <c r="E1657" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1658" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1658" t="s">
+        <v>641</v>
+      </c>
+      <c r="C1658" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1658">
+        <v>4</v>
+      </c>
+      <c r="E1658" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1659" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1659" t="s">
+        <v>255</v>
+      </c>
+      <c r="C1659" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1659">
+        <v>2</v>
+      </c>
+      <c r="E1659" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1660" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1660" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1660" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1660">
+        <v>1</v>
+      </c>
+      <c r="E1660" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1661" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1661" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1661" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1661">
+        <v>2</v>
+      </c>
+      <c r="E1661" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1662" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1662" t="s">
+        <v>585</v>
+      </c>
+      <c r="C1662" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1662">
+        <v>3</v>
+      </c>
+      <c r="E1662" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1663" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1663" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1663" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1663">
+        <v>5</v>
+      </c>
+      <c r="E1663" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1664" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1664" t="s">
+        <v>261</v>
+      </c>
+      <c r="C1664" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1664">
+        <v>2</v>
+      </c>
+      <c r="E1664" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1665" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1665" t="s">
+        <v>262</v>
+      </c>
+      <c r="C1665" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1665">
+        <v>3</v>
+      </c>
+      <c r="E1665" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1666" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1666" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1666" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1666">
+        <v>3</v>
+      </c>
+      <c r="E1666" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1667" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1667" t="s">
+        <v>264</v>
+      </c>
+      <c r="C1667" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1667">
+        <v>2</v>
+      </c>
+      <c r="E1667" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1668" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1668" t="s">
+        <v>644</v>
+      </c>
+      <c r="C1668" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1668">
+        <v>5</v>
+      </c>
+      <c r="E1668" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1669" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1669" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1669" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1669">
+        <v>1</v>
+      </c>
+      <c r="E1669" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1670" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1670" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1670" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1670">
+        <v>5</v>
+      </c>
+      <c r="E1670" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1671" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1671" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1671" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1671">
+        <v>2</v>
+      </c>
+      <c r="E1671" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1672" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1672" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1672" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1672">
+        <v>2</v>
+      </c>
+      <c r="E1672" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1673" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1673" t="s">
+        <v>645</v>
+      </c>
+      <c r="C1673" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1673">
+        <v>4</v>
+      </c>
+      <c r="E1673" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1674" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1674" t="s">
+        <v>274</v>
+      </c>
+      <c r="C1674" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1674">
+        <v>5</v>
+      </c>
+      <c r="E1674" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1675" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1675" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1675" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1675">
+        <v>2</v>
+      </c>
+      <c r="E1675" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1676" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1676" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1676" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1676">
+        <v>5</v>
+      </c>
+      <c r="E1676" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1677" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1677" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1677" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1677">
+        <v>2</v>
+      </c>
+      <c r="E1677" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1678" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1678" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1678" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1678">
+        <v>4</v>
+      </c>
+      <c r="E1678" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1679" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1679" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1679" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1679">
+        <v>5</v>
+      </c>
+      <c r="E1679" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1680" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1680" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1680" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1680">
+        <v>2</v>
+      </c>
+      <c r="E1680" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1681" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1681" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1681" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1681">
+        <v>5</v>
+      </c>
+      <c r="E1681" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1682" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1682" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1682" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1682">
+        <v>5</v>
+      </c>
+      <c r="E1682" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1683" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1683" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1683" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1683">
+        <v>4</v>
+      </c>
+      <c r="E1683" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1684" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1684" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1684" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1684">
+        <v>3</v>
+      </c>
+      <c r="E1684" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1685" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1685" t="s">
+        <v>285</v>
+      </c>
+      <c r="C1685" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1685">
+        <v>5</v>
+      </c>
+      <c r="E1685" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1686" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1686" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1686" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1686">
+        <v>2</v>
+      </c>
+      <c r="E1686" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1687" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1687" t="s">
+        <v>649</v>
+      </c>
+      <c r="C1687" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1687">
+        <v>5</v>
+      </c>
+      <c r="E1687" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1688" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1688" t="s">
+        <v>650</v>
+      </c>
+      <c r="C1688" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1688">
+        <v>5</v>
+      </c>
+      <c r="E1688" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1689" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1689" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1689" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1689">
+        <v>2</v>
+      </c>
+      <c r="E1689" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1690" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1690" t="s">
+        <v>699</v>
+      </c>
+      <c r="C1690" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1690">
+        <v>2</v>
+      </c>
+      <c r="E1690" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1691" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1691" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1691" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1691">
+        <v>2</v>
+      </c>
+      <c r="E1691" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1692" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1692" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1692" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1692">
+        <v>5</v>
+      </c>
+      <c r="E1692" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1693" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1693" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1693" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1693">
+        <v>2</v>
+      </c>
+      <c r="E1693" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1694" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1694" t="s">
+        <v>294</v>
+      </c>
+      <c r="C1694" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1694">
+        <v>2</v>
+      </c>
+      <c r="E1694" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1695" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1695" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1695" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1695">
+        <v>3</v>
+      </c>
+      <c r="E1695" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1696" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1696" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1696" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1696">
+        <v>5</v>
+      </c>
+      <c r="E1696" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1697" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1697" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1697" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1697">
+        <v>2</v>
+      </c>
+      <c r="E1697" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1698" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1698" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1698" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1698">
+        <v>3</v>
+      </c>
+      <c r="E1698" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1699" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1699" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1699" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1699">
+        <v>5</v>
+      </c>
+      <c r="E1699" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="1700" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1700" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1700" t="s">
+        <v>701</v>
+      </c>
+      <c r="C1700" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1700">
+        <v>4</v>
+      </c>
+      <c r="E1700" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="1701" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1701" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1701" t="s">
+        <v>741</v>
+      </c>
+      <c r="C1701" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1701">
+        <v>3</v>
+      </c>
+      <c r="E1701" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1702" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1702" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1702" t="s">
+        <v>302</v>
+      </c>
+      <c r="C1702" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1702">
+        <v>2</v>
+      </c>
+      <c r="E1702" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1703" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1703" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1703" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1703" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1703">
+        <v>3</v>
+      </c>
+      <c r="E1703" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="1704" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1704" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1704" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1704" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1704">
+        <v>3</v>
+      </c>
+      <c r="E1704" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1705" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1705" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1705" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1705" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1705">
+        <v>1</v>
+      </c>
+      <c r="E1705" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1706" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1706" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1706" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1706" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1706">
+        <v>3</v>
+      </c>
+      <c r="E1706" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="1707" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1707" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1707" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1707" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1707">
+        <v>1</v>
+      </c>
+      <c r="E1707" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1708" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1708" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="B1708" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1708" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1708">
+        <v>2</v>
+      </c>
+      <c r="E1708" t="s">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adding April Metric Data
</commit_message>
<xml_diff>
--- a/Tutor_Concerns.xlsx
+++ b/Tutor_Concerns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tylerharrington/Desktop/Revolution Prep/FL_Dashboards/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B7E57B33-0637-4E4B-971B-1977EBD743D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{232BE9F0-233F-EE40-8ACB-91CCFD870F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17860" xr2:uid="{92DEE1D6-509C-344A-AA8F-D8DD2317BD81}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="6833" uniqueCount="744">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="7769" uniqueCount="808">
   <si>
     <t>Tutor Name</t>
   </si>
@@ -2268,6 +2268,198 @@
   </si>
   <si>
     <t>2/22/26 - 3/21/26</t>
+  </si>
+  <si>
+    <t>Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>Breanna Lowe</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>Denise Jefferson</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % Sessions on Time &lt; 90%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%</t>
+  </si>
+  <si>
+    <t>Emma Claire Everett</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Gene Costa</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Avg. NPS Score &lt; 8; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>Jason Pranaitis</t>
+  </si>
+  <si>
+    <t>Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; Avg. NPS Score &lt; 8; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Katie Soller</t>
+  </si>
+  <si>
+    <t>Kayleigh Puliafico</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Sessions on Time &lt; 85%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 85%; Prep Time % &gt; 15%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>Lilly Kellogg</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % Sessions on Time &lt; 90%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>Qualondra Kimber</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>% of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>Savannah Padgett</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 70%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Avg. NPS Score &lt; 8</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%</t>
+  </si>
+  <si>
+    <t>Tim Page</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 90%; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Diff M2M % of Active Students with Progress Updates Completed in last 2 months &lt; -20%</t>
+  </si>
+  <si>
+    <t>% to Availability Target &lt; 90%; % Parent Updates &lt; 85%; Prep Time % &gt; 15%; Diff M2M % to Availability Target &lt; -10% and % to Availability Target &lt; 95%</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 85%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 50%; Prep Time % &gt; 15%; Diff M2M Prep Time % &gt; 10%; Bottom 10% in % to Delivery Target for tier</t>
+  </si>
+  <si>
+    <t>% Parent Updates &lt; 90%; Ratio of PPW Events with Attached PPW &lt; 1/2; % of Active Students with Progress Updates Completed in last 2 months &lt; 60%; Prep Time % &gt; 15%; Diff M2M % to Delivery Target &lt; -20% and % to Delivery Target &lt; 85%</t>
+  </si>
+  <si>
+    <t>3/22/26 - 4/18/26</t>
   </si>
 </sst>
 </file>
@@ -3137,7 +3329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDA4CB91-83C8-694D-BBCD-170E9881DA10}">
-  <dimension ref="A1:E1708"/>
+  <dimension ref="A1:E1942"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
@@ -32179,6 +32371,3984 @@
         <v>121</v>
       </c>
     </row>
+    <row r="1709" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1709" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1709" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1709" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1709">
+        <v>5</v>
+      </c>
+      <c r="E1709" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="1710" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1710" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1710" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1710" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1710">
+        <v>2</v>
+      </c>
+      <c r="E1710" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1711" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1711" t="s">
+        <v>657</v>
+      </c>
+      <c r="C1711" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1711">
+        <v>5</v>
+      </c>
+      <c r="E1711" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="1712" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1712" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1712" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1712" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1712">
+        <v>5</v>
+      </c>
+      <c r="E1712" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="1713" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1713" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1713" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1713" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1713">
+        <v>2</v>
+      </c>
+      <c r="E1713" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1714" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1714" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1714" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1714" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1714">
+        <v>5</v>
+      </c>
+      <c r="E1714" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1715" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1715" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1715" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1715" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1715">
+        <v>4</v>
+      </c>
+      <c r="E1715" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="1716" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1716" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1716" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1716" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1716">
+        <v>5</v>
+      </c>
+      <c r="E1716" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="1717" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1717" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1717" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1717" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1717">
+        <v>5</v>
+      </c>
+      <c r="E1717" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="1718" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1718" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1718" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1718" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1718">
+        <v>5</v>
+      </c>
+      <c r="E1718" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="1719" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1719" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1719" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1719" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1719">
+        <v>5</v>
+      </c>
+      <c r="E1719" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="1720" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1720" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1720" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1720" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1720">
+        <v>5</v>
+      </c>
+      <c r="E1720" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1721" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1721" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1721" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1721" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1721">
+        <v>3</v>
+      </c>
+      <c r="E1721" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1722" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1722" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1722" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1722" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1722">
+        <v>3</v>
+      </c>
+      <c r="E1722" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="1723" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1723" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1723" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1723" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1723">
+        <v>3</v>
+      </c>
+      <c r="E1723" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="1724" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1724" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1724" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1724" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1724">
+        <v>5</v>
+      </c>
+      <c r="E1724" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1725" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1725" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1725" t="s">
+        <v>663</v>
+      </c>
+      <c r="C1725" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1725">
+        <v>5</v>
+      </c>
+      <c r="E1725" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="1726" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1726" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1726" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1726" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1726">
+        <v>3</v>
+      </c>
+      <c r="E1726" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="1727" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1727" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1727" t="s">
+        <v>709</v>
+      </c>
+      <c r="C1727" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1727">
+        <v>5</v>
+      </c>
+      <c r="E1727" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="1728" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1728" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1728" t="s">
+        <v>607</v>
+      </c>
+      <c r="C1728" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1728">
+        <v>5</v>
+      </c>
+      <c r="E1728" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="1729" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1729" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1729" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1729" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1729">
+        <v>2</v>
+      </c>
+      <c r="E1729" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="1730" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1730" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1730" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1730" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1730">
+        <v>5</v>
+      </c>
+      <c r="E1730" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="1731" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1731" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1731" t="s">
+        <v>534</v>
+      </c>
+      <c r="C1731" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1731">
+        <v>5</v>
+      </c>
+      <c r="E1731" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="1732" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1732" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1732" t="s">
+        <v>665</v>
+      </c>
+      <c r="C1732" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1732">
+        <v>5</v>
+      </c>
+      <c r="E1732" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="1733" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1733" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1733" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1733" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1733">
+        <v>5</v>
+      </c>
+      <c r="E1733" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1734" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1734" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1734" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1734" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1734">
+        <v>3</v>
+      </c>
+      <c r="E1734" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1735" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1735" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1735" t="s">
+        <v>609</v>
+      </c>
+      <c r="C1735" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1735">
+        <v>1</v>
+      </c>
+      <c r="E1735" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1736" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1736" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1736" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1736" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1736">
+        <v>4</v>
+      </c>
+      <c r="E1736" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1737" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1737" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1737" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1737" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1737">
+        <v>5</v>
+      </c>
+      <c r="E1737" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="1738" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1738" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1738" t="s">
+        <v>747</v>
+      </c>
+      <c r="C1738" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1738">
+        <v>3</v>
+      </c>
+      <c r="E1738" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1739" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1739" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1739" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1739" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1739">
+        <v>2</v>
+      </c>
+      <c r="E1739" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1740" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1740" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1740" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1740" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1740">
+        <v>1</v>
+      </c>
+      <c r="E1740" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1741" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1741" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1741" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1741" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1741">
+        <v>5</v>
+      </c>
+      <c r="E1741" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="1742" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1742" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1742" t="s">
+        <v>710</v>
+      </c>
+      <c r="C1742" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1742">
+        <v>5</v>
+      </c>
+      <c r="E1742" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1743" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1743" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1743" t="s">
+        <v>610</v>
+      </c>
+      <c r="C1743" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1743">
+        <v>2</v>
+      </c>
+      <c r="E1743" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1744" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1744" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1744" t="s">
+        <v>465</v>
+      </c>
+      <c r="C1744" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1744">
+        <v>3</v>
+      </c>
+      <c r="E1744" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1745" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1745" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1745" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1745" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1745">
+        <v>5</v>
+      </c>
+      <c r="E1745" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1746" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1746" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1746" t="s">
+        <v>711</v>
+      </c>
+      <c r="C1746" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1746">
+        <v>5</v>
+      </c>
+      <c r="E1746" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="1747" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1747" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1747" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1747" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1747">
+        <v>5</v>
+      </c>
+      <c r="E1747" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="1748" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1748" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1748" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1748" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1748">
+        <v>5</v>
+      </c>
+      <c r="E1748" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1749" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1749" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1749" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1749" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1749">
+        <v>4</v>
+      </c>
+      <c r="E1749" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="1750" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1750" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1750" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1750" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1750">
+        <v>4</v>
+      </c>
+      <c r="E1750" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="1751" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1751" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1751" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1751" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1751">
+        <v>5</v>
+      </c>
+      <c r="E1751" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="1752" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1752" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1752" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1752" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1752">
+        <v>5</v>
+      </c>
+      <c r="E1752" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1753" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1753" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1753" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1753" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1753">
+        <v>5</v>
+      </c>
+      <c r="E1753" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="1754" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1754" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1754" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1754" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1754">
+        <v>2</v>
+      </c>
+      <c r="E1754" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1755" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1755" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1755" t="s">
+        <v>668</v>
+      </c>
+      <c r="C1755" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1755">
+        <v>5</v>
+      </c>
+      <c r="E1755" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="1756" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1756" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1756" t="s">
+        <v>541</v>
+      </c>
+      <c r="C1756" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1756">
+        <v>2</v>
+      </c>
+      <c r="E1756" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1757" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1757" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1757" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1757" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1757">
+        <v>5</v>
+      </c>
+      <c r="E1757" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1758" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1758" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1758" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1758" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1758">
+        <v>5</v>
+      </c>
+      <c r="E1758" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1759" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1759" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1759" t="s">
+        <v>471</v>
+      </c>
+      <c r="C1759" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1759">
+        <v>5</v>
+      </c>
+      <c r="E1759" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1760" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1760" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1760" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1760" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1760">
+        <v>3</v>
+      </c>
+      <c r="E1760" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="1761" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1761" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1761" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1761" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1761">
+        <v>2</v>
+      </c>
+      <c r="E1761" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1762" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1762" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1762" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1762" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1762">
+        <v>5</v>
+      </c>
+      <c r="E1762" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1763" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1763" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1763" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1763" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1763">
+        <v>5</v>
+      </c>
+      <c r="E1763" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="1764" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1764" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1764" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1764" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1764">
+        <v>2</v>
+      </c>
+      <c r="E1764" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1765" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1765" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1765" t="s">
+        <v>713</v>
+      </c>
+      <c r="C1765" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1765">
+        <v>5</v>
+      </c>
+      <c r="E1765" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="1766" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1766" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1766" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1766" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1766">
+        <v>2</v>
+      </c>
+      <c r="E1766" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1767" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1767" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1767" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1767" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1767">
+        <v>5</v>
+      </c>
+      <c r="E1767" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1768" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1768" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1768" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1768" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1768">
+        <v>5</v>
+      </c>
+      <c r="E1768" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1769" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1769" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1769" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1769" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1769">
+        <v>5</v>
+      </c>
+      <c r="E1769" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1770" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1770" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1770" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1770" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1770">
+        <v>5</v>
+      </c>
+      <c r="E1770" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="1771" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1771" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1771" t="s">
+        <v>100</v>
+      </c>
+      <c r="C1771" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1771">
+        <v>4</v>
+      </c>
+      <c r="E1771" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="1772" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1772" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1772" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1772" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1772">
+        <v>5</v>
+      </c>
+      <c r="E1772" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="1773" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1773" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1773" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1773" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1773">
+        <v>3</v>
+      </c>
+      <c r="E1773" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="1774" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1774" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1774" t="s">
+        <v>757</v>
+      </c>
+      <c r="C1774" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1774">
+        <v>3</v>
+      </c>
+      <c r="E1774" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1775" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1775" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1775" t="s">
+        <v>544</v>
+      </c>
+      <c r="C1775" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1775">
+        <v>4</v>
+      </c>
+      <c r="E1775" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="1776" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1776" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1776" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1776" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1776">
+        <v>5</v>
+      </c>
+      <c r="E1776" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1777" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1777" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1777" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1777" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1777">
+        <v>3</v>
+      </c>
+      <c r="E1777" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="1778" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1778" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1778" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1778" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1778">
+        <v>5</v>
+      </c>
+      <c r="E1778" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="1779" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1779" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1779" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1779" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1779">
+        <v>5</v>
+      </c>
+      <c r="E1779" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1780" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1780" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1780" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1780" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1780">
+        <v>2</v>
+      </c>
+      <c r="E1780" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1781" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1781" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1781" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1781" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1781">
+        <v>5</v>
+      </c>
+      <c r="E1781" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="1782" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1782" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1782" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1782" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1782">
+        <v>3</v>
+      </c>
+      <c r="E1782" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="1783" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1783" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1783" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1783" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1783">
+        <v>5</v>
+      </c>
+      <c r="E1783" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="1784" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1784" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1784" t="s">
+        <v>116</v>
+      </c>
+      <c r="C1784" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1784">
+        <v>5</v>
+      </c>
+      <c r="E1784" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1785" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1785" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1785" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1785" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1785">
+        <v>5</v>
+      </c>
+      <c r="E1785" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="1786" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1786" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1786" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1786" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1786">
+        <v>5</v>
+      </c>
+      <c r="E1786" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="1787" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1787" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1787" t="s">
+        <v>762</v>
+      </c>
+      <c r="C1787" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1787">
+        <v>3</v>
+      </c>
+      <c r="E1787" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1788" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1788" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1788" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1788" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1788">
+        <v>5</v>
+      </c>
+      <c r="E1788" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="1789" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1789" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1789" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1789" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1789">
+        <v>5</v>
+      </c>
+      <c r="E1789" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1790" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1790" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1790" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1790" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1790">
+        <v>5</v>
+      </c>
+      <c r="E1790" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1791" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1791" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1791" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1791" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1791">
+        <v>5</v>
+      </c>
+      <c r="E1791" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="1792" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1792" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1792" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1792" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1792">
+        <v>2</v>
+      </c>
+      <c r="E1792" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1793" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1793" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1793" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1793" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1793">
+        <v>5</v>
+      </c>
+      <c r="E1793" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1794" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1794" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1794" t="s">
+        <v>764</v>
+      </c>
+      <c r="C1794" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1794">
+        <v>3</v>
+      </c>
+      <c r="E1794" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1795" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1795" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1795" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1795" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1795">
+        <v>2</v>
+      </c>
+      <c r="E1795" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="1796" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1796" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1796" t="s">
+        <v>720</v>
+      </c>
+      <c r="C1796" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1796">
+        <v>5</v>
+      </c>
+      <c r="E1796" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="1797" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1797" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1797" t="s">
+        <v>141</v>
+      </c>
+      <c r="C1797" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1797">
+        <v>5</v>
+      </c>
+      <c r="E1797" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1798" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1798" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1798" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1798" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1798">
+        <v>3</v>
+      </c>
+      <c r="E1798" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1799" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1799" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1799" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1799">
+        <v>5</v>
+      </c>
+      <c r="E1799" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1800" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1800" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1800" t="s">
+        <v>673</v>
+      </c>
+      <c r="C1800" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1800">
+        <v>4</v>
+      </c>
+      <c r="E1800" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1801" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1801" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1801" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1801">
+        <v>5</v>
+      </c>
+      <c r="E1801" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="1802" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1802" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1802" t="s">
+        <v>675</v>
+      </c>
+      <c r="C1802" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1802">
+        <v>2</v>
+      </c>
+      <c r="E1802" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="1803" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1803" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1803" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1803" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1803">
+        <v>5</v>
+      </c>
+      <c r="E1803" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1804" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1804" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1804" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1804" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1804">
+        <v>5</v>
+      </c>
+      <c r="E1804" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="1805" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1805" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1805" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1805" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1805">
+        <v>4</v>
+      </c>
+      <c r="E1805" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="1806" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1806" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1806" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1806" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1806">
+        <v>2</v>
+      </c>
+      <c r="E1806" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1807" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1807" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1807" t="s">
+        <v>150</v>
+      </c>
+      <c r="C1807" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1807">
+        <v>2</v>
+      </c>
+      <c r="E1807" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="1808" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1808" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1808" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1808" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1808">
+        <v>4</v>
+      </c>
+      <c r="E1808" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="1809" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1809" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1809" t="s">
+        <v>769</v>
+      </c>
+      <c r="C1809" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1809">
+        <v>3</v>
+      </c>
+      <c r="E1809" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1810" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1810" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1810" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1810" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1810">
+        <v>5</v>
+      </c>
+      <c r="E1810" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1811" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1811" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1811" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1811" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1811">
+        <v>3</v>
+      </c>
+      <c r="E1811" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="1812" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1812" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1812" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1812" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1812">
+        <v>5</v>
+      </c>
+      <c r="E1812" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1813" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1813" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1813" t="s">
+        <v>158</v>
+      </c>
+      <c r="C1813" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1813">
+        <v>2</v>
+      </c>
+      <c r="E1813" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="1814" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1814" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1814" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1814" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1814">
+        <v>2</v>
+      </c>
+      <c r="E1814" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="1815" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1815" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1815" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1815" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1815">
+        <v>3</v>
+      </c>
+      <c r="E1815" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1816" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1816" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1816" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1816" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1816">
+        <v>5</v>
+      </c>
+      <c r="E1816" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1817" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1817" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1817" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1817" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1817">
+        <v>2</v>
+      </c>
+      <c r="E1817" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1818" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1818" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1818" t="s">
+        <v>678</v>
+      </c>
+      <c r="C1818" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1818">
+        <v>5</v>
+      </c>
+      <c r="E1818" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="1819" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1819" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1819" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1819" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1819">
+        <v>2</v>
+      </c>
+      <c r="E1819" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1820" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1820" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1820" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1820" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1820">
+        <v>5</v>
+      </c>
+      <c r="E1820" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1821" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1821" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1821" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1821" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1821">
+        <v>5</v>
+      </c>
+      <c r="E1821" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1822" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1822" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1822" t="s">
+        <v>722</v>
+      </c>
+      <c r="C1822" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1822">
+        <v>5</v>
+      </c>
+      <c r="E1822" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="1823" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1823" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1823" t="s">
+        <v>680</v>
+      </c>
+      <c r="C1823" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1823">
+        <v>5</v>
+      </c>
+      <c r="E1823" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1824" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1824" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1824" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1824" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1824">
+        <v>3</v>
+      </c>
+      <c r="E1824" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="1825" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1825" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1825" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1825" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1825">
+        <v>1</v>
+      </c>
+      <c r="E1825" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1826" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1826" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1826" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1826" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1826">
+        <v>5</v>
+      </c>
+      <c r="E1826" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="1827" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1827" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1827" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1827" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1827">
+        <v>5</v>
+      </c>
+      <c r="E1827" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1828" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1828" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1828" t="s">
+        <v>559</v>
+      </c>
+      <c r="C1828" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1828">
+        <v>5</v>
+      </c>
+      <c r="E1828" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1829" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1829" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1829" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1829" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1829">
+        <v>2</v>
+      </c>
+      <c r="E1829" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1830" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1830" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1830" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1830" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1830">
+        <v>5</v>
+      </c>
+      <c r="E1830" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="1831" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1831" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1831" t="s">
+        <v>178</v>
+      </c>
+      <c r="C1831" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1831">
+        <v>1</v>
+      </c>
+      <c r="E1831" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1832" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1832" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1832" t="s">
+        <v>723</v>
+      </c>
+      <c r="C1832" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1832">
+        <v>5</v>
+      </c>
+      <c r="E1832" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="1833" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1833" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1833" t="s">
+        <v>682</v>
+      </c>
+      <c r="C1833" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1833">
+        <v>5</v>
+      </c>
+      <c r="E1833" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="1834" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1834" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1834" t="s">
+        <v>179</v>
+      </c>
+      <c r="C1834" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1834">
+        <v>5</v>
+      </c>
+      <c r="E1834" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1835" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1835" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1835" t="s">
+        <v>560</v>
+      </c>
+      <c r="C1835" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1835">
+        <v>3</v>
+      </c>
+      <c r="E1835" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="1836" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1836" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1836" t="s">
+        <v>724</v>
+      </c>
+      <c r="C1836" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1836">
+        <v>5</v>
+      </c>
+      <c r="E1836" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1837" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1837" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1837" t="s">
+        <v>181</v>
+      </c>
+      <c r="C1837" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1837">
+        <v>5</v>
+      </c>
+      <c r="E1837" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1838" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1838" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1838" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1838" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1838">
+        <v>5</v>
+      </c>
+      <c r="E1838" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1839" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1839" t="s">
+        <v>775</v>
+      </c>
+      <c r="C1839" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1839">
+        <v>1</v>
+      </c>
+      <c r="E1839" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1840" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1840" t="s">
+        <v>776</v>
+      </c>
+      <c r="C1840" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1840">
+        <v>3</v>
+      </c>
+      <c r="E1840" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1841" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1841" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1841" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1841">
+        <v>5</v>
+      </c>
+      <c r="E1841" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1842" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1842" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1842" t="s">
+        <v>626</v>
+      </c>
+      <c r="C1842" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1842">
+        <v>5</v>
+      </c>
+      <c r="E1842" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1843" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1843" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1843" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1843" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1843">
+        <v>5</v>
+      </c>
+      <c r="E1843" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="1844" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1844" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1844" t="s">
+        <v>189</v>
+      </c>
+      <c r="C1844" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1844">
+        <v>5</v>
+      </c>
+      <c r="E1844" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="1845" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1845" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1845" t="s">
+        <v>191</v>
+      </c>
+      <c r="C1845" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1845">
+        <v>5</v>
+      </c>
+      <c r="E1845" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1846" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1846" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1846" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1846" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1846">
+        <v>5</v>
+      </c>
+      <c r="E1846" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="1847" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1847" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1847" t="s">
+        <v>779</v>
+      </c>
+      <c r="C1847" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1847">
+        <v>1</v>
+      </c>
+      <c r="E1847" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1848" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1848" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1848" t="s">
+        <v>195</v>
+      </c>
+      <c r="C1848" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1848">
+        <v>5</v>
+      </c>
+      <c r="E1848" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1849" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1849" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1849" t="s">
+        <v>197</v>
+      </c>
+      <c r="C1849" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1849">
+        <v>4</v>
+      </c>
+      <c r="E1849" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="1850" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1850" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1850" t="s">
+        <v>198</v>
+      </c>
+      <c r="C1850" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1850">
+        <v>4</v>
+      </c>
+      <c r="E1850" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1851" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1851" t="s">
+        <v>685</v>
+      </c>
+      <c r="C1851" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1851">
+        <v>2</v>
+      </c>
+      <c r="E1851" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1852" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1852" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1852" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1852" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1852">
+        <v>5</v>
+      </c>
+      <c r="E1852" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="1853" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1853" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1853" t="s">
+        <v>204</v>
+      </c>
+      <c r="C1853" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1853">
+        <v>5</v>
+      </c>
+      <c r="E1853" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="1854" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1854" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1854" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1854" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1854">
+        <v>2</v>
+      </c>
+      <c r="E1854" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1855" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1855" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1855" t="s">
+        <v>207</v>
+      </c>
+      <c r="C1855" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1855">
+        <v>1</v>
+      </c>
+      <c r="E1855" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1856" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1856" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1856" t="s">
+        <v>686</v>
+      </c>
+      <c r="C1856" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1856">
+        <v>3</v>
+      </c>
+      <c r="E1856" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="1857" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1857" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1857" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1857" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1857">
+        <v>5</v>
+      </c>
+      <c r="E1857" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1858" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1858" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1858" t="s">
+        <v>211</v>
+      </c>
+      <c r="C1858" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1858">
+        <v>5</v>
+      </c>
+      <c r="E1858" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1859" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1859" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1859" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1859" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1859">
+        <v>1</v>
+      </c>
+      <c r="E1859" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1860" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1860" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1860" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1860" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1860">
+        <v>4</v>
+      </c>
+      <c r="E1860" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1861" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1861" t="s">
+        <v>215</v>
+      </c>
+      <c r="C1861" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1861">
+        <v>5</v>
+      </c>
+      <c r="E1861" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="1862" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1862" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1862" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1862" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1862">
+        <v>5</v>
+      </c>
+      <c r="E1862" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="1863" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1863" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1863" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1863" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1863">
+        <v>5</v>
+      </c>
+      <c r="E1863" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="1864" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1864" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1864" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1864" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1864">
+        <v>5</v>
+      </c>
+      <c r="E1864" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1865" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1865" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1865" t="s">
+        <v>691</v>
+      </c>
+      <c r="C1865" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1865">
+        <v>5</v>
+      </c>
+      <c r="E1865" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="1866" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1866" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1866" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1866" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1866">
+        <v>1</v>
+      </c>
+      <c r="E1866" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1867" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1867" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1867" t="s">
+        <v>223</v>
+      </c>
+      <c r="C1867" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1867">
+        <v>2</v>
+      </c>
+      <c r="E1867" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1868" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1868" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1868" t="s">
+        <v>224</v>
+      </c>
+      <c r="C1868" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1868">
+        <v>1</v>
+      </c>
+      <c r="E1868" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1869" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1869" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1869" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1869" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1869">
+        <v>1</v>
+      </c>
+      <c r="E1869" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1870" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1870" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1870" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1870" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1870">
+        <v>5</v>
+      </c>
+      <c r="E1870" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="1871" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1871" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1871" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1871" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1871">
+        <v>4</v>
+      </c>
+      <c r="E1871" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="1872" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1872" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1872" t="s">
+        <v>633</v>
+      </c>
+      <c r="C1872" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1872">
+        <v>4</v>
+      </c>
+      <c r="E1872" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1873" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1873" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1873" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1873">
+        <v>5</v>
+      </c>
+      <c r="E1873" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1874" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1874" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1874" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1874">
+        <v>2</v>
+      </c>
+      <c r="E1874" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1875" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1875" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1875" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1875">
+        <v>5</v>
+      </c>
+      <c r="E1875" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1876" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1876" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1876" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1876">
+        <v>5</v>
+      </c>
+      <c r="E1876" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1877" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1877" t="s">
+        <v>238</v>
+      </c>
+      <c r="C1877" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1877">
+        <v>5</v>
+      </c>
+      <c r="E1877" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1878" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1878" t="s">
+        <v>239</v>
+      </c>
+      <c r="C1878" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1878">
+        <v>5</v>
+      </c>
+      <c r="E1878" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1879" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1879" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1879" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1879">
+        <v>5</v>
+      </c>
+      <c r="E1879" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1880" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1880" t="s">
+        <v>242</v>
+      </c>
+      <c r="C1880" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1880">
+        <v>5</v>
+      </c>
+      <c r="E1880" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1881" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1881" t="s">
+        <v>729</v>
+      </c>
+      <c r="C1881" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1881">
+        <v>5</v>
+      </c>
+      <c r="E1881" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1882" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1882" t="s">
+        <v>637</v>
+      </c>
+      <c r="C1882" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1882">
+        <v>2</v>
+      </c>
+      <c r="E1882" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1883" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1883" t="s">
+        <v>730</v>
+      </c>
+      <c r="C1883" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1883">
+        <v>5</v>
+      </c>
+      <c r="E1883" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1884" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1884" t="s">
+        <v>244</v>
+      </c>
+      <c r="C1884" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1884">
+        <v>5</v>
+      </c>
+      <c r="E1884" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1885" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1885" t="s">
+        <v>247</v>
+      </c>
+      <c r="C1885" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1885">
+        <v>5</v>
+      </c>
+      <c r="E1885" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1886" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1886" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1886" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1886">
+        <v>5</v>
+      </c>
+      <c r="E1886" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1887" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1887" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1887" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1887">
+        <v>5</v>
+      </c>
+      <c r="E1887" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1888" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1888" t="s">
+        <v>252</v>
+      </c>
+      <c r="C1888" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1888">
+        <v>4</v>
+      </c>
+      <c r="E1888" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1889" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1889" t="s">
+        <v>791</v>
+      </c>
+      <c r="C1889" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1889">
+        <v>3</v>
+      </c>
+      <c r="E1889" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1890" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1890" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1890" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1890">
+        <v>5</v>
+      </c>
+      <c r="E1890" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1891" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1891" t="s">
+        <v>640</v>
+      </c>
+      <c r="C1891" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1891">
+        <v>5</v>
+      </c>
+      <c r="E1891" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1892" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1892" t="s">
+        <v>641</v>
+      </c>
+      <c r="C1892" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1892">
+        <v>4</v>
+      </c>
+      <c r="E1892" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1893" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1893" t="s">
+        <v>255</v>
+      </c>
+      <c r="C1893" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1893">
+        <v>5</v>
+      </c>
+      <c r="E1893" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1894" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1894" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1894" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1894">
+        <v>1</v>
+      </c>
+      <c r="E1894" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1895" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1895" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1895" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1895">
+        <v>3</v>
+      </c>
+      <c r="E1895" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1896" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1896" t="s">
+        <v>585</v>
+      </c>
+      <c r="C1896" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1896">
+        <v>3</v>
+      </c>
+      <c r="E1896" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1897" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1897" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1897" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1897">
+        <v>5</v>
+      </c>
+      <c r="E1897" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1898" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1898" t="s">
+        <v>261</v>
+      </c>
+      <c r="C1898" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1898">
+        <v>5</v>
+      </c>
+      <c r="E1898" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1899" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1899" t="s">
+        <v>262</v>
+      </c>
+      <c r="C1899" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1899">
+        <v>5</v>
+      </c>
+      <c r="E1899" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1900" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1900" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1900" t="s">
+        <v>263</v>
+      </c>
+      <c r="C1900" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1900">
+        <v>5</v>
+      </c>
+      <c r="E1900" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="1901" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1901" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1901" t="s">
+        <v>264</v>
+      </c>
+      <c r="C1901" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1901">
+        <v>5</v>
+      </c>
+      <c r="E1901" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1902" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1902" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1902" t="s">
+        <v>644</v>
+      </c>
+      <c r="C1902" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1902">
+        <v>4</v>
+      </c>
+      <c r="E1902" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="1903" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1903" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1903" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1903" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1903">
+        <v>5</v>
+      </c>
+      <c r="E1903" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="1904" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1904" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1904" t="s">
+        <v>270</v>
+      </c>
+      <c r="C1904" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1904">
+        <v>5</v>
+      </c>
+      <c r="E1904" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="1905" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1905" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1905" t="s">
+        <v>796</v>
+      </c>
+      <c r="C1905" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1905">
+        <v>1</v>
+      </c>
+      <c r="E1905" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1906" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1906" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1906" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1906" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1906">
+        <v>5</v>
+      </c>
+      <c r="E1906" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="1907" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1907" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1907" t="s">
+        <v>274</v>
+      </c>
+      <c r="C1907" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1907">
+        <v>5</v>
+      </c>
+      <c r="E1907" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="1908" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1908" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1908" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1908" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1908">
+        <v>3</v>
+      </c>
+      <c r="E1908" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="1909" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1909" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1909" t="s">
+        <v>276</v>
+      </c>
+      <c r="C1909" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1909">
+        <v>5</v>
+      </c>
+      <c r="E1909" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="1910" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1910" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1910" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1910" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1910">
+        <v>2</v>
+      </c>
+      <c r="E1910" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1911" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1911" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1911" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1911" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1911">
+        <v>2</v>
+      </c>
+      <c r="E1911" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="1912" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1912" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1912" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1912" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1912">
+        <v>5</v>
+      </c>
+      <c r="E1912" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="1913" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1913" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1913" t="s">
+        <v>280</v>
+      </c>
+      <c r="C1913" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1913">
+        <v>5</v>
+      </c>
+      <c r="E1913" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1914" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1914" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1914" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1914" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1914">
+        <v>5</v>
+      </c>
+      <c r="E1914" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="1915" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1915" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1915" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1915" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1915">
+        <v>5</v>
+      </c>
+      <c r="E1915" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="1916" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1916" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1916" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1916" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1916">
+        <v>3</v>
+      </c>
+      <c r="E1916" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="1917" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1917" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1917" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1917" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1917">
+        <v>5</v>
+      </c>
+      <c r="E1917" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="1918" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1918" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1918" t="s">
+        <v>285</v>
+      </c>
+      <c r="C1918" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1918">
+        <v>5</v>
+      </c>
+      <c r="E1918" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="1919" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1919" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1919" t="s">
+        <v>286</v>
+      </c>
+      <c r="C1919" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1919">
+        <v>2</v>
+      </c>
+      <c r="E1919" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1920" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1920" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1920" t="s">
+        <v>649</v>
+      </c>
+      <c r="C1920" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1920">
+        <v>2</v>
+      </c>
+      <c r="E1920" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1921" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1921" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1921" t="s">
+        <v>650</v>
+      </c>
+      <c r="C1921" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1921">
+        <v>5</v>
+      </c>
+      <c r="E1921" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="1922" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1922" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1922" t="s">
+        <v>288</v>
+      </c>
+      <c r="C1922" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1922">
+        <v>5</v>
+      </c>
+      <c r="E1922" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="1923" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1923" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1923" t="s">
+        <v>699</v>
+      </c>
+      <c r="C1923" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1923">
+        <v>5</v>
+      </c>
+      <c r="E1923" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="1924" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1924" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1924" t="s">
+        <v>801</v>
+      </c>
+      <c r="C1924" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1924">
+        <v>3</v>
+      </c>
+      <c r="E1924" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="1925" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1925" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1925" t="s">
+        <v>289</v>
+      </c>
+      <c r="C1925" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1925">
+        <v>2</v>
+      </c>
+      <c r="E1925" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1926" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1926" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1926" t="s">
+        <v>290</v>
+      </c>
+      <c r="C1926" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1926">
+        <v>5</v>
+      </c>
+      <c r="E1926" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="1927" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1927" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1927" t="s">
+        <v>292</v>
+      </c>
+      <c r="C1927" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1927">
+        <v>5</v>
+      </c>
+      <c r="E1927" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="1928" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1928" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1928" t="s">
+        <v>294</v>
+      </c>
+      <c r="C1928" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1928">
+        <v>5</v>
+      </c>
+      <c r="E1928" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="1929" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1929" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1929" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1929" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1929">
+        <v>5</v>
+      </c>
+      <c r="E1929" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="1930" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1930" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1930" t="s">
+        <v>297</v>
+      </c>
+      <c r="C1930" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1930">
+        <v>5</v>
+      </c>
+      <c r="E1930" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="1931" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1931" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1931" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1931" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1931">
+        <v>2</v>
+      </c>
+      <c r="E1931" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="1932" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1932" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1932" t="s">
+        <v>299</v>
+      </c>
+      <c r="C1932" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1932">
+        <v>2</v>
+      </c>
+      <c r="E1932" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1933" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1933" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1933" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1933" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1933">
+        <v>5</v>
+      </c>
+      <c r="E1933" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="1934" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1934" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1934" t="s">
+        <v>701</v>
+      </c>
+      <c r="C1934" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1934">
+        <v>5</v>
+      </c>
+      <c r="E1934" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="1935" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1935" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1935" t="s">
+        <v>741</v>
+      </c>
+      <c r="C1935" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1935">
+        <v>5</v>
+      </c>
+      <c r="E1935" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="1936" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1936" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1936" t="s">
+        <v>302</v>
+      </c>
+      <c r="C1936" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1936">
+        <v>4</v>
+      </c>
+      <c r="E1936" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="1937" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1937" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1937" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1937" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1937">
+        <v>5</v>
+      </c>
+      <c r="E1937" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1938" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1938" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1938" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1938" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1938">
+        <v>5</v>
+      </c>
+      <c r="E1938" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="1939" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1939" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1939" t="s">
+        <v>306</v>
+      </c>
+      <c r="C1939" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1939">
+        <v>5</v>
+      </c>
+      <c r="E1939" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1940" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1940" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1940" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1940" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1940">
+        <v>1</v>
+      </c>
+      <c r="E1940" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1941" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1941" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1941" t="s">
+        <v>310</v>
+      </c>
+      <c r="C1941" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1941">
+        <v>2</v>
+      </c>
+      <c r="E1941" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="1942" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1942" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="B1942" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1942" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1942">
+        <v>5</v>
+      </c>
+      <c r="E1942" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>